<commit_message>
Data files updated upto 6 aug 2026
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/order_files/Mapped_Expired_OrderBook_Equity_5aug26_Wed.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/order_files/Mapped_Expired_OrderBook_Equity_5aug26_Wed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\order_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D2147D-91EB-442C-81F3-B011EA0793DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1F7563-B4A1-49D0-8A69-4844C7A719A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -693,7 +693,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -727,23 +727,22 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="22" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1106,7 +1105,7 @@
         <v>9</v>
       </c>
       <c r="G2">
-        <f>((E2-I2)/E2)*100</f>
+        <f t="shared" ref="G2:G33" si="0">((E2-I2)/E2)*100</f>
         <v>-24.936126724578436</v>
       </c>
       <c r="H2" s="9" t="s">
@@ -1116,7 +1115,7 @@
         <v>4890</v>
       </c>
       <c r="K2" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B2, $C$2:$C$979, C2, $D$2:$D$979, D2, $E$2:$E$979, E2) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="K2:K33" si="1">IF(COUNTIFS( $B$2:$B$979, B2, $C$2:$C$979, C2, $D$2:$D$979, D2, $E$2:$E$979, E2) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -1140,7 +1139,7 @@
         <v>9</v>
       </c>
       <c r="G3">
-        <f>((E3-I3)/E3)*100</f>
+        <f t="shared" si="0"/>
         <v>-23.837209302325583</v>
       </c>
       <c r="H3" s="9" t="s">
@@ -1150,7 +1149,7 @@
         <v>2556</v>
       </c>
       <c r="K3" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B3, $C$2:$C$979, C3, $D$2:$D$979, D3, $E$2:$E$979, E3) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1174,7 +1173,7 @@
         <v>9</v>
       </c>
       <c r="G4">
-        <f>((E4-I4)/E4)*100</f>
+        <f t="shared" si="0"/>
         <v>-21.823617339312406</v>
       </c>
       <c r="H4" s="9" t="s">
@@ -1184,7 +1183,7 @@
         <v>4890</v>
       </c>
       <c r="K4" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B4, $C$2:$C$979, C4, $D$2:$D$979, D4, $E$2:$E$979, E4) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1208,7 +1207,7 @@
         <v>9</v>
       </c>
       <c r="G5">
-        <f>((E5-I5)/E5)*100</f>
+        <f t="shared" si="0"/>
         <v>-18.898809523809522</v>
       </c>
       <c r="H5" s="9" t="s">
@@ -1218,31 +1217,31 @@
         <v>399.5</v>
       </c>
       <c r="K5" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B5, $C$2:$C$979, C5, $D$2:$D$979, D5, $E$2:$E$979, E5) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="18" t="s">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="18">
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6">
         <v>2</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6">
         <v>2164</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" t="s">
         <v>9</v>
       </c>
       <c r="G6">
-        <f>((E6-I6)/E6)*100</f>
+        <f t="shared" si="0"/>
         <v>-18.11460258780037</v>
       </c>
       <c r="H6" s="9" t="s">
@@ -1252,7 +1251,7 @@
         <v>2556</v>
       </c>
       <c r="K6" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B6, $C$2:$C$979, C6, $D$2:$D$979, D6, $E$2:$E$979, E6) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1276,7 +1275,7 @@
         <v>9</v>
       </c>
       <c r="G7">
-        <f>((E7-I7)/E7)*100</f>
+        <f t="shared" si="0"/>
         <v>-17.435158501440924</v>
       </c>
       <c r="H7" s="9" t="s">
@@ -1286,7 +1285,7 @@
         <v>4890</v>
       </c>
       <c r="K7" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B7, $C$2:$C$979, C7, $D$2:$D$979, D7, $E$2:$E$979, E7) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1310,7 +1309,7 @@
         <v>9</v>
       </c>
       <c r="G8">
-        <f>((E8-I8)/E8)*100</f>
+        <f t="shared" si="0"/>
         <v>-16.533523537803134</v>
       </c>
       <c r="H8" s="9" t="s">
@@ -1320,7 +1319,7 @@
         <v>816.9</v>
       </c>
       <c r="K8" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B8, $C$2:$C$979, C8, $D$2:$D$979, D8, $E$2:$E$979, E8) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1344,7 +1343,7 @@
         <v>9</v>
       </c>
       <c r="G9">
-        <f>((E9-I9)/E9)*100</f>
+        <f t="shared" si="0"/>
         <v>-16.50872817955112</v>
       </c>
       <c r="H9" s="9" t="s">
@@ -1354,7 +1353,7 @@
         <v>467.2</v>
       </c>
       <c r="K9" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B9, $C$2:$C$979, C9, $D$2:$D$979, D9, $E$2:$E$979, E9) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1378,7 +1377,7 @@
         <v>9</v>
       </c>
       <c r="G10">
-        <f>((E10-I10)/E10)*100</f>
+        <f t="shared" si="0"/>
         <v>-13.494318181818182</v>
       </c>
       <c r="H10" s="9" t="s">
@@ -1388,31 +1387,31 @@
         <v>399.5</v>
       </c>
       <c r="K10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B10, $C$2:$C$979, C10, $D$2:$D$979, D10, $E$2:$E$979, E10) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="18" t="s">
+      <c r="A11" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="18">
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11">
         <v>1</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11">
         <v>2264</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" t="s">
         <v>9</v>
       </c>
       <c r="G11">
-        <f>((E11-I11)/E11)*100</f>
+        <f t="shared" si="0"/>
         <v>-12.897526501766784</v>
       </c>
       <c r="H11" s="9" t="s">
@@ -1422,7 +1421,7 @@
         <v>2556</v>
       </c>
       <c r="K11" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B11, $C$2:$C$979, C11, $D$2:$D$979, D11, $E$2:$E$979, E11) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1446,7 +1445,7 @@
         <v>9</v>
       </c>
       <c r="G12">
-        <f>((E12-I12)/E12)*100</f>
+        <f t="shared" si="0"/>
         <v>-12.0807453416149</v>
       </c>
       <c r="H12" s="9" t="s">
@@ -1456,7 +1455,7 @@
         <v>360.9</v>
       </c>
       <c r="K12" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B12, $C$2:$C$979, C12, $D$2:$D$979, D12, $E$2:$E$979, E12) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1480,7 +1479,7 @@
         <v>9</v>
       </c>
       <c r="G13">
-        <f>((E13-I13)/E13)*100</f>
+        <f t="shared" si="0"/>
         <v>-12.060625604643658</v>
       </c>
       <c r="H13" s="9" t="s">
@@ -1490,7 +1489,7 @@
         <v>34.75</v>
       </c>
       <c r="K13" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B13, $C$2:$C$979, C13, $D$2:$D$979, D13, $E$2:$E$979, E13) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1514,7 +1513,7 @@
         <v>9</v>
       </c>
       <c r="G14">
-        <f>((E14-I14)/E14)*100</f>
+        <f t="shared" si="0"/>
         <v>-12.053162236480294</v>
       </c>
       <c r="H14" s="9" t="s">
@@ -1524,7 +1523,7 @@
         <v>4890</v>
       </c>
       <c r="K14" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B14, $C$2:$C$979, C14, $D$2:$D$979, D14, $E$2:$E$979, E14) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1548,7 +1547,7 @@
         <v>9</v>
       </c>
       <c r="G15">
-        <f>((E15-I15)/E15)*100</f>
+        <f t="shared" si="0"/>
         <v>-11.517341040462428</v>
       </c>
       <c r="H15" s="9" t="s">
@@ -1558,7 +1557,7 @@
         <v>7717</v>
       </c>
       <c r="K15" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B15, $C$2:$C$979, C15, $D$2:$D$979, D15, $E$2:$E$979, E15) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1582,7 +1581,7 @@
         <v>9</v>
       </c>
       <c r="G16">
-        <f>((E16-I16)/E16)*100</f>
+        <f t="shared" si="0"/>
         <v>-11.503579952267302</v>
       </c>
       <c r="H16" s="9" t="s">
@@ -1592,31 +1591,31 @@
         <v>467.2</v>
       </c>
       <c r="K16" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B16, $C$2:$C$979, C16, $D$2:$D$979, D16, $E$2:$E$979, E16) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="18" t="s">
+      <c r="A17" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="18">
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17">
         <v>2</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17">
         <v>4410</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="F17" t="s">
         <v>9</v>
       </c>
       <c r="G17">
-        <f>((E17-I17)/E17)*100</f>
+        <f t="shared" si="0"/>
         <v>-10.884353741496598</v>
       </c>
       <c r="H17" s="9" t="s">
@@ -1626,7 +1625,7 @@
         <v>4890</v>
       </c>
       <c r="K17" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B17, $C$2:$C$979, C17, $D$2:$D$979, D17, $E$2:$E$979, E17) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1650,7 +1649,7 @@
         <v>9</v>
       </c>
       <c r="G18">
-        <f>((E18-I18)/E18)*100</f>
+        <f t="shared" si="0"/>
         <v>-10.513715710723201</v>
       </c>
       <c r="H18" s="9" t="s">
@@ -1660,7 +1659,7 @@
         <v>4431.6000000000004</v>
       </c>
       <c r="K18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B18, $C$2:$C$979, C18, $D$2:$D$979, D18, $E$2:$E$979, E18) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1684,7 +1683,7 @@
         <v>9</v>
       </c>
       <c r="G19">
-        <f>((E19-I19)/E19)*100</f>
+        <f t="shared" si="0"/>
         <v>-10.366972477064214</v>
       </c>
       <c r="H19" s="9" t="s">
@@ -1694,7 +1693,7 @@
         <v>360.9</v>
       </c>
       <c r="K19" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B19, $C$2:$C$979, C19, $D$2:$D$979, D19, $E$2:$E$979, E19) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1718,7 +1717,7 @@
         <v>9</v>
       </c>
       <c r="G20">
-        <f>((E20-I20)/E20)*100</f>
+        <f t="shared" si="0"/>
         <v>-10.258215962441312</v>
       </c>
       <c r="H20" s="9" t="s">
@@ -1728,7 +1727,7 @@
         <v>939.4</v>
       </c>
       <c r="K20" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B20, $C$2:$C$979, C20, $D$2:$D$979, D20, $E$2:$E$979, E20) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1752,7 +1751,7 @@
         <v>9</v>
       </c>
       <c r="G21">
-        <f>((E21-I21)/E21)*100</f>
+        <f t="shared" si="0"/>
         <v>-9.7080291970802861</v>
       </c>
       <c r="H21" s="9" t="s">
@@ -1762,7 +1761,7 @@
         <v>450.9</v>
       </c>
       <c r="K21" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B21, $C$2:$C$979, C21, $D$2:$D$979, D21, $E$2:$E$979, E21) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1786,7 +1785,7 @@
         <v>9</v>
       </c>
       <c r="G22">
-        <f>((E22-I22)/E22)*100</f>
+        <f t="shared" si="0"/>
         <v>-9.5418326693227051</v>
       </c>
       <c r="H22" s="9" t="s">
@@ -1796,7 +1795,7 @@
         <v>274.95</v>
       </c>
       <c r="K22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B22, $C$2:$C$979, C22, $D$2:$D$979, D22, $E$2:$E$979, E22) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1820,7 +1819,7 @@
         <v>9</v>
       </c>
       <c r="G23">
-        <f>((E23-I23)/E23)*100</f>
+        <f t="shared" si="0"/>
         <v>-9.2325581395348806</v>
       </c>
       <c r="H23" s="9" t="s">
@@ -1830,7 +1829,7 @@
         <v>939.4</v>
       </c>
       <c r="K23" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B23, $C$2:$C$979, C23, $D$2:$D$979, D23, $E$2:$E$979, E23) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1854,7 +1853,7 @@
         <v>9</v>
       </c>
       <c r="G24">
-        <f>((E24-I24)/E24)*100</f>
+        <f t="shared" si="0"/>
         <v>-9.1530054644808754</v>
       </c>
       <c r="H24" s="9" t="s">
@@ -1864,7 +1863,7 @@
         <v>399.5</v>
       </c>
       <c r="K24" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B24, $C$2:$C$979, C24, $D$2:$D$979, D24, $E$2:$E$979, E24) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1888,7 +1887,7 @@
         <v>9</v>
       </c>
       <c r="G25">
-        <f>((E25-I25)/E25)*100</f>
+        <f t="shared" si="0"/>
         <v>-9.1527093596059199</v>
       </c>
       <c r="H25" s="9" t="s">
@@ -1898,7 +1897,7 @@
         <v>4431.6000000000004</v>
       </c>
       <c r="K25" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B25, $C$2:$C$979, C25, $D$2:$D$979, D25, $E$2:$E$979, E25) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1922,7 +1921,7 @@
         <v>9</v>
       </c>
       <c r="G26">
-        <f>((E26-I26)/E26)*100</f>
+        <f t="shared" si="0"/>
         <v>-9.0332326283987854</v>
       </c>
       <c r="H26" s="9" t="s">
@@ -1932,7 +1931,7 @@
         <v>360.9</v>
       </c>
       <c r="K26" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B26, $C$2:$C$979, C26, $D$2:$D$979, D26, $E$2:$E$979, E26) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1956,7 +1955,7 @@
         <v>9</v>
       </c>
       <c r="G27">
-        <f>((E27-I27)/E27)*100</f>
+        <f t="shared" si="0"/>
         <v>-8.6330049261083772</v>
       </c>
       <c r="H27" s="9" t="s">
@@ -1966,7 +1965,7 @@
         <v>882.1</v>
       </c>
       <c r="K27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B27, $C$2:$C$979, C27, $D$2:$D$979, D27, $E$2:$E$979, E27) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -1990,7 +1989,7 @@
         <v>9</v>
       </c>
       <c r="G28">
-        <f>((E28-I28)/E28)*100</f>
+        <f t="shared" si="0"/>
         <v>-8.3754512635379008</v>
       </c>
       <c r="H28" s="9" t="s">
@@ -2000,7 +1999,7 @@
         <v>300.2</v>
       </c>
       <c r="K28" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B28, $C$2:$C$979, C28, $D$2:$D$979, D28, $E$2:$E$979, E28) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2024,7 +2023,7 @@
         <v>9</v>
       </c>
       <c r="G29">
-        <f>((E29-I29)/E29)*100</f>
+        <f t="shared" si="0"/>
         <v>-8.1707317073170653</v>
       </c>
       <c r="H29" s="9" t="s">
@@ -2034,7 +2033,7 @@
         <v>1153.0999999999999</v>
       </c>
       <c r="K29" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B29, $C$2:$C$979, C29, $D$2:$D$979, D29, $E$2:$E$979, E29) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2058,7 +2057,7 @@
         <v>9</v>
       </c>
       <c r="G30">
-        <f>((E30-I30)/E30)*100</f>
+        <f t="shared" si="0"/>
         <v>-8.0580865603644654</v>
       </c>
       <c r="H30" s="9" t="s">
@@ -2068,7 +2067,7 @@
         <v>948.75</v>
       </c>
       <c r="K30" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B30, $C$2:$C$979, C30, $D$2:$D$979, D30, $E$2:$E$979, E30) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2092,7 +2091,7 @@
         <v>9</v>
       </c>
       <c r="G31">
-        <f>((E31-I31)/E31)*100</f>
+        <f t="shared" si="0"/>
         <v>-8.0525414049114783</v>
       </c>
       <c r="H31" s="9" t="s">
@@ -2102,7 +2101,7 @@
         <v>1892</v>
       </c>
       <c r="K31" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B31, $C$2:$C$979, C31, $D$2:$D$979, D31, $E$2:$E$979, E31) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2126,7 +2125,7 @@
         <v>9</v>
       </c>
       <c r="G32">
-        <f>((E32-I32)/E32)*100</f>
+        <f t="shared" si="0"/>
         <v>-7.8248175182481834</v>
       </c>
       <c r="H32" s="9" t="s">
@@ -2136,7 +2135,7 @@
         <v>4431.6000000000004</v>
       </c>
       <c r="K32" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B32, $C$2:$C$979, C32, $D$2:$D$979, D32, $E$2:$E$979, E32) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2160,7 +2159,7 @@
         <v>9</v>
       </c>
       <c r="G33">
-        <f>((E33-I33)/E33)*100</f>
+        <f t="shared" si="0"/>
         <v>-7.731343283582083</v>
       </c>
       <c r="H33" s="9" t="s">
@@ -2170,7 +2169,7 @@
         <v>360.9</v>
       </c>
       <c r="K33" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B33, $C$2:$C$979, C33, $D$2:$D$979, D33, $E$2:$E$979, E33) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2194,7 +2193,7 @@
         <v>9</v>
       </c>
       <c r="G34">
-        <f>((E34-I34)/E34)*100</f>
+        <f t="shared" ref="G34:G65" si="2">((E34-I34)/E34)*100</f>
         <v>-7.6869806094182831</v>
       </c>
       <c r="H34" s="9" t="s">
@@ -2204,7 +2203,7 @@
         <v>3110</v>
       </c>
       <c r="K34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B34, $C$2:$C$979, C34, $D$2:$D$979, D34, $E$2:$E$979, E34) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="K34:K65" si="3">IF(COUNTIFS( $B$2:$B$979, B34, $C$2:$C$979, C34, $D$2:$D$979, D34, $E$2:$E$979, E34) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -2228,7 +2227,7 @@
         <v>9</v>
       </c>
       <c r="G35">
-        <f>((E35-I35)/E35)*100</f>
+        <f t="shared" si="2"/>
         <v>-7.6329787234042561</v>
       </c>
       <c r="H35" s="9" t="s">
@@ -2238,7 +2237,7 @@
         <v>4047</v>
       </c>
       <c r="K35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B35, $C$2:$C$979, C35, $D$2:$D$979, D35, $E$2:$E$979, E35) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2262,7 +2261,7 @@
         <v>9</v>
       </c>
       <c r="G36">
-        <f>((E36-I36)/E36)*100</f>
+        <f t="shared" si="2"/>
         <v>-7.5135135135135176</v>
       </c>
       <c r="H36" s="9" t="s">
@@ -2272,7 +2271,7 @@
         <v>119.34</v>
       </c>
       <c r="K36" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B36, $C$2:$C$979, C36, $D$2:$D$979, D36, $E$2:$E$979, E36) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2296,7 +2295,7 @@
         <v>9</v>
       </c>
       <c r="G37">
-        <f>((E37-I37)/E37)*100</f>
+        <f t="shared" si="2"/>
         <v>-7.2501110617503253</v>
       </c>
       <c r="H37" s="9" t="s">
@@ -2306,7 +2305,7 @@
         <v>2414.1999999999998</v>
       </c>
       <c r="K37" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B37, $C$2:$C$979, C37, $D$2:$D$979, D37, $E$2:$E$979, E37) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2330,7 +2329,7 @@
         <v>9</v>
       </c>
       <c r="G38">
-        <f>((E38-I38)/E38)*100</f>
+        <f t="shared" si="2"/>
         <v>-7.0919881305637906</v>
       </c>
       <c r="H38" s="9" t="s">
@@ -2340,7 +2339,7 @@
         <v>360.9</v>
       </c>
       <c r="K38" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B38, $C$2:$C$979, C38, $D$2:$D$979, D38, $E$2:$E$979, E38) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2364,7 +2363,7 @@
         <v>9</v>
       </c>
       <c r="G39">
-        <f>((E39-I39)/E39)*100</f>
+        <f t="shared" si="2"/>
         <v>-7.03125</v>
       </c>
       <c r="H39" s="9" t="s">
@@ -2374,7 +2373,7 @@
         <v>685</v>
       </c>
       <c r="K39" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B39, $C$2:$C$979, C39, $D$2:$D$979, D39, $E$2:$E$979, E39) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2398,7 +2397,7 @@
         <v>9</v>
       </c>
       <c r="G40">
-        <f>((E40-I40)/E40)*100</f>
+        <f t="shared" si="2"/>
         <v>-7.0229681978798588</v>
       </c>
       <c r="H40" s="9" t="s">
@@ -2408,7 +2407,7 @@
         <v>1211.5</v>
       </c>
       <c r="K40" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B40, $C$2:$C$979, C40, $D$2:$D$979, D40, $E$2:$E$979, E40) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2432,7 +2431,7 @@
         <v>9</v>
       </c>
       <c r="G41">
-        <f>((E41-I41)/E41)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.9554030874785511</v>
       </c>
       <c r="H41" s="9" t="s">
@@ -2442,7 +2441,7 @@
         <v>1247.0999999999999</v>
       </c>
       <c r="K41" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B41, $C$2:$C$979, C41, $D$2:$D$979, D41, $E$2:$E$979, E41) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2466,7 +2465,7 @@
         <v>9</v>
       </c>
       <c r="G42">
-        <f>((E42-I42)/E42)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.90178571428571</v>
       </c>
       <c r="H42" s="9" t="s">
@@ -2476,7 +2475,7 @@
         <v>598.65</v>
       </c>
       <c r="K42" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B42, $C$2:$C$979, C42, $D$2:$D$979, D42, $E$2:$E$979, E42) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2500,7 +2499,7 @@
         <v>9</v>
       </c>
       <c r="G43">
-        <f>((E43-I43)/E43)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.8327402135231283</v>
       </c>
       <c r="H43" s="9" t="s">
@@ -2510,7 +2509,7 @@
         <v>300.2</v>
       </c>
       <c r="K43" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B43, $C$2:$C$979, C43, $D$2:$D$979, D43, $E$2:$E$979, E43) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2534,7 +2533,7 @@
         <v>9</v>
       </c>
       <c r="G44">
-        <f>((E44-I44)/E44)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.7527308838133067</v>
       </c>
       <c r="H44" s="9" t="s">
@@ -2544,7 +2543,7 @@
         <v>1075</v>
       </c>
       <c r="K44" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B44, $C$2:$C$979, C44, $D$2:$D$979, D44, $E$2:$E$979, E44) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2568,7 +2567,7 @@
         <v>9</v>
       </c>
       <c r="G45">
-        <f>((E45-I45)/E45)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.5079365079365052</v>
       </c>
       <c r="H45" s="9" t="s">
@@ -2578,7 +2577,7 @@
         <v>939.4</v>
       </c>
       <c r="K45" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B45, $C$2:$C$979, C45, $D$2:$D$979, D45, $E$2:$E$979, E45) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2602,7 +2601,7 @@
         <v>9</v>
       </c>
       <c r="G46">
-        <f>((E46-I46)/E46)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.2630890052356047</v>
       </c>
       <c r="H46" s="9" t="s">
@@ -2612,7 +2611,7 @@
         <v>811.85</v>
       </c>
       <c r="K46" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B46, $C$2:$C$979, C46, $D$2:$D$979, D46, $E$2:$E$979, E46) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2636,7 +2635,7 @@
         <v>9</v>
       </c>
       <c r="G47">
-        <f>((E47-I47)/E47)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.2598632298790147</v>
       </c>
       <c r="H47" s="9" t="s">
@@ -2646,7 +2645,7 @@
         <v>202</v>
       </c>
       <c r="K47" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B47, $C$2:$C$979, C47, $D$2:$D$979, D47, $E$2:$E$979, E47) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2670,7 +2669,7 @@
         <v>9</v>
       </c>
       <c r="G48">
-        <f>((E48-I48)/E48)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.2204724409448815</v>
       </c>
       <c r="H48" s="9" t="s">
@@ -2680,7 +2679,7 @@
         <v>4047</v>
       </c>
       <c r="K48" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B48, $C$2:$C$979, C48, $D$2:$D$979, D48, $E$2:$E$979, E48) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2704,7 +2703,7 @@
         <v>9</v>
       </c>
       <c r="G49">
-        <f>((E49-I49)/E49)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.0858143607705779</v>
       </c>
       <c r="H49" s="9" t="s">
@@ -2714,7 +2713,7 @@
         <v>1211.5</v>
       </c>
       <c r="K49" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B49, $C$2:$C$979, C49, $D$2:$D$979, D49, $E$2:$E$979, E49) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2738,7 +2737,7 @@
         <v>9</v>
       </c>
       <c r="G50">
-        <f>((E50-I50)/E50)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.084656084656082</v>
       </c>
       <c r="H50" s="9" t="s">
@@ -2748,31 +2747,31 @@
         <v>360.9</v>
       </c>
       <c r="K50" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B50, $C$2:$C$979, C50, $D$2:$D$979, D50, $E$2:$E$979, E50) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A51" s="18" t="s">
+      <c r="A51" t="s">
         <v>71</v>
       </c>
-      <c r="B51" s="18" t="s">
+      <c r="B51" t="s">
         <v>57</v>
       </c>
-      <c r="C51" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D51" s="18">
+      <c r="C51" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" s="18">
+      <c r="E51">
         <v>3310</v>
       </c>
-      <c r="F51" s="18" t="s">
+      <c r="F51" t="s">
         <v>9</v>
       </c>
       <c r="G51">
-        <f>((E51-I51)/E51)*100</f>
+        <f t="shared" si="2"/>
         <v>-6.0725075528700909</v>
       </c>
       <c r="H51" s="9" t="s">
@@ -2782,31 +2781,31 @@
         <v>3511</v>
       </c>
       <c r="K51" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B51, $C$2:$C$979, C51, $D$2:$D$979, D51, $E$2:$E$979, E51) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A52" s="18" t="s">
+      <c r="A52" t="s">
         <v>91</v>
       </c>
-      <c r="B52" s="18" t="s">
+      <c r="B52" t="s">
         <v>92</v>
       </c>
-      <c r="C52" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D52" s="18">
+      <c r="C52" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52">
         <v>1</v>
       </c>
-      <c r="E52" s="18">
+      <c r="E52">
         <v>13552</v>
       </c>
-      <c r="F52" s="18" t="s">
+      <c r="F52" t="s">
         <v>9</v>
       </c>
       <c r="G52">
-        <f>((E52-I52)/E52)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.9622195985832347</v>
       </c>
       <c r="H52" s="9" t="s">
@@ -2816,31 +2815,31 @@
         <v>14360</v>
       </c>
       <c r="K52" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B52, $C$2:$C$979, C52, $D$2:$D$979, D52, $E$2:$E$979, E52) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="18" t="s">
+      <c r="A53" t="s">
         <v>71</v>
       </c>
-      <c r="B53" s="18" t="s">
+      <c r="B53" t="s">
         <v>80</v>
       </c>
-      <c r="C53" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D53" s="18">
+      <c r="C53" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53">
         <v>5</v>
       </c>
-      <c r="E53" s="18">
+      <c r="E53">
         <v>2938</v>
       </c>
-      <c r="F53" s="18" t="s">
+      <c r="F53" t="s">
         <v>9</v>
       </c>
       <c r="G53">
-        <f>((E53-I53)/E53)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.8543226684819611</v>
       </c>
       <c r="H53" s="9" t="s">
@@ -2850,7 +2849,7 @@
         <v>3110</v>
       </c>
       <c r="K53" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B53, $C$2:$C$979, C53, $D$2:$D$979, D53, $E$2:$E$979, E53) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2874,7 +2873,7 @@
         <v>9</v>
       </c>
       <c r="G54">
-        <f>((E54-I54)/E54)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.7692307692307692</v>
       </c>
       <c r="H54" s="9" t="s">
@@ -2884,7 +2883,7 @@
         <v>948.75</v>
       </c>
       <c r="K54" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B54, $C$2:$C$979, C54, $D$2:$D$979, D54, $E$2:$E$979, E54) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2908,7 +2907,7 @@
         <v>9</v>
       </c>
       <c r="G55">
-        <f>((E55-I55)/E55)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.6657963446475197</v>
       </c>
       <c r="H55" s="9" t="s">
@@ -2918,7 +2917,7 @@
         <v>4047</v>
       </c>
       <c r="K55" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B55, $C$2:$C$979, C55, $D$2:$D$979, D55, $E$2:$E$979, E55) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2942,7 +2941,7 @@
         <v>9</v>
       </c>
       <c r="G56">
-        <f>((E56-I56)/E56)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.6435643564356468</v>
       </c>
       <c r="H56" s="9" t="s">
@@ -2952,7 +2951,7 @@
         <v>213.4</v>
       </c>
       <c r="K56" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B56, $C$2:$C$979, C56, $D$2:$D$979, D56, $E$2:$E$979, E56) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2976,7 +2975,7 @@
         <v>9</v>
       </c>
       <c r="G57">
-        <f>((E57-I57)/E57)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.514354066985649</v>
       </c>
       <c r="H57" s="9" t="s">
@@ -2986,31 +2985,31 @@
         <v>882.1</v>
       </c>
       <c r="K57" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B57, $C$2:$C$979, C57, $D$2:$D$979, D57, $E$2:$E$979, E57) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A58" s="18" t="s">
+      <c r="A58" t="s">
         <v>71</v>
       </c>
-      <c r="B58" s="18" t="s">
+      <c r="B58" t="s">
         <v>83</v>
       </c>
-      <c r="C58" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58" s="18">
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58">
         <v>1</v>
       </c>
-      <c r="E58" s="18">
+      <c r="E58">
         <v>4206</v>
       </c>
-      <c r="F58" s="18" t="s">
+      <c r="F58" t="s">
         <v>9</v>
       </c>
       <c r="G58">
-        <f>((E58-I58)/E58)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.3637660485021481</v>
       </c>
       <c r="H58" s="9" t="s">
@@ -3020,7 +3019,7 @@
         <v>4431.6000000000004</v>
       </c>
       <c r="K58" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B58, $C$2:$C$979, C58, $D$2:$D$979, D58, $E$2:$E$979, E58) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3044,7 +3043,7 @@
         <v>9</v>
       </c>
       <c r="G59">
-        <f>((E59-I59)/E59)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.262529832935563</v>
       </c>
       <c r="H59" s="9" t="s">
@@ -3054,7 +3053,7 @@
         <v>882.1</v>
       </c>
       <c r="K59" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B59, $C$2:$C$979, C59, $D$2:$D$979, D59, $E$2:$E$979, E59) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3078,7 +3077,7 @@
         <v>9</v>
       </c>
       <c r="G60">
-        <f>((E60-I60)/E60)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.1649305555555554</v>
       </c>
       <c r="H60" s="9" t="s">
@@ -3088,7 +3087,7 @@
         <v>1211.5</v>
       </c>
       <c r="K60" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B60, $C$2:$C$979, C60, $D$2:$D$979, D60, $E$2:$E$979, E60) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3112,7 +3111,7 @@
         <v>9</v>
       </c>
       <c r="G61">
-        <f>((E61-I61)/E61)*100</f>
+        <f t="shared" si="2"/>
         <v>-5.0312155710613249</v>
       </c>
       <c r="H61" s="9" t="s">
@@ -3122,31 +3121,31 @@
         <v>143</v>
       </c>
       <c r="K61" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B61, $C$2:$C$979, C61, $D$2:$D$979, D61, $E$2:$E$979, E61) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A62" s="18" t="s">
+      <c r="A62" t="s">
         <v>61</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" t="s">
         <v>62</v>
       </c>
-      <c r="C62" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D62" s="18">
+      <c r="C62" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62">
         <v>15</v>
       </c>
-      <c r="E62" s="18">
+      <c r="E62">
         <v>4415</v>
       </c>
-      <c r="F62" s="18" t="s">
+      <c r="F62" t="s">
         <v>9</v>
       </c>
       <c r="G62">
-        <f>((E62-I62)/E62)*100</f>
+        <f t="shared" si="2"/>
         <v>-4.992072480181192</v>
       </c>
       <c r="H62" s="9" t="s">
@@ -3156,7 +3155,7 @@
         <v>4635.3999999999996</v>
       </c>
       <c r="K62" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B62, $C$2:$C$979, C62, $D$2:$D$979, D62, $E$2:$E$979, E62) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3180,7 +3179,7 @@
         <v>9</v>
       </c>
       <c r="G63">
-        <f>((E63-I63)/E63)*100</f>
+        <f t="shared" si="2"/>
         <v>-4.9747474747474669</v>
       </c>
       <c r="H63" s="9" t="s">
@@ -3190,7 +3189,7 @@
         <v>1247.0999999999999</v>
       </c>
       <c r="K63" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B63, $C$2:$C$979, C63, $D$2:$D$979, D63, $E$2:$E$979, E63) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3214,7 +3213,7 @@
         <v>9</v>
       </c>
       <c r="G64">
-        <f>((E64-I64)/E64)*100</f>
+        <f t="shared" si="2"/>
         <v>-4.9650349650349614</v>
       </c>
       <c r="H64" s="9" t="s">
@@ -3224,7 +3223,7 @@
         <v>300.2</v>
       </c>
       <c r="K64" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B64, $C$2:$C$979, C64, $D$2:$D$979, D64, $E$2:$E$979, E64) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3248,7 +3247,7 @@
         <v>9</v>
       </c>
       <c r="G65">
-        <f>((E65-I65)/E65)*100</f>
+        <f t="shared" si="2"/>
         <v>-4.953319502074689</v>
       </c>
       <c r="H65" s="9" t="s">
@@ -3258,7 +3257,7 @@
         <v>4047</v>
       </c>
       <c r="K65" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B65, $C$2:$C$979, C65, $D$2:$D$979, D65, $E$2:$E$979, E65) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3282,7 +3281,7 @@
         <v>9</v>
       </c>
       <c r="G66">
-        <f>((E66-I66)/E66)*100</f>
+        <f t="shared" ref="G66:G97" si="4">((E66-I66)/E66)*100</f>
         <v>-4.9253731343283587</v>
       </c>
       <c r="H66" s="9" t="s">
@@ -3292,7 +3291,7 @@
         <v>1054.5</v>
       </c>
       <c r="K66" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B66, $C$2:$C$979, C66, $D$2:$D$979, D66, $E$2:$E$979, E66) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="K66:K97" si="5">IF(COUNTIFS( $B$2:$B$979, B66, $C$2:$C$979, C66, $D$2:$D$979, D66, $E$2:$E$979, E66) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -3316,7 +3315,7 @@
         <v>9</v>
       </c>
       <c r="G67">
-        <f>((E67-I67)/E67)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.9127906976744118</v>
       </c>
       <c r="H67" s="9" t="s">
@@ -3326,7 +3325,7 @@
         <v>360.9</v>
       </c>
       <c r="K67" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B67, $C$2:$C$979, C67, $D$2:$D$979, D67, $E$2:$E$979, E67) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3350,7 +3349,7 @@
         <v>9</v>
       </c>
       <c r="G68">
-        <f>((E68-I68)/E68)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.8028714676390152</v>
       </c>
       <c r="H68" s="9" t="s">
@@ -3360,7 +3359,7 @@
         <v>18395</v>
       </c>
       <c r="K68" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B68, $C$2:$C$979, C68, $D$2:$D$979, D68, $E$2:$E$979, E68) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3384,7 +3383,7 @@
         <v>9</v>
       </c>
       <c r="G69">
-        <f>((E69-I69)/E69)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.7949336550060426</v>
       </c>
       <c r="H69" s="9" t="s">
@@ -3394,7 +3393,7 @@
         <v>34.75</v>
       </c>
       <c r="K69" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B69, $C$2:$C$979, C69, $D$2:$D$979, D69, $E$2:$E$979, E69) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3418,7 +3417,7 @@
         <v>9</v>
       </c>
       <c r="G70">
-        <f>((E70-I70)/E70)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.700854700854701</v>
       </c>
       <c r="H70" s="9" t="s">
@@ -3428,7 +3427,7 @@
         <v>735</v>
       </c>
       <c r="K70" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B70, $C$2:$C$979, C70, $D$2:$D$979, D70, $E$2:$E$979, E70) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3452,7 +3451,7 @@
         <v>9</v>
       </c>
       <c r="G71">
-        <f>((E71-I71)/E71)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.4940476190476186</v>
       </c>
       <c r="H71" s="9" t="s">
@@ -3462,7 +3461,7 @@
         <v>3511</v>
       </c>
       <c r="K71" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B71, $C$2:$C$979, C71, $D$2:$D$979, D71, $E$2:$E$979, E71) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3486,7 +3485,7 @@
         <v>9</v>
       </c>
       <c r="G72">
-        <f>((E72-I72)/E72)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.3496985357450475</v>
       </c>
       <c r="H72" s="9" t="s">
@@ -3496,7 +3495,7 @@
         <v>1211.5</v>
       </c>
       <c r="K72" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B72, $C$2:$C$979, C72, $D$2:$D$979, D72, $E$2:$E$979, E72) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3520,7 +3519,7 @@
         <v>9</v>
       </c>
       <c r="G73">
-        <f>((E73-I73)/E73)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.1503523884103366</v>
       </c>
       <c r="H73" s="9" t="s">
@@ -3530,7 +3529,7 @@
         <v>1330</v>
       </c>
       <c r="K73" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B73, $C$2:$C$979, C73, $D$2:$D$979, D73, $E$2:$E$979, E73) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3554,7 +3553,7 @@
         <v>9</v>
       </c>
       <c r="G74">
-        <f>((E74-I74)/E74)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.0895061728395063</v>
       </c>
       <c r="H74" s="9" t="s">
@@ -3564,7 +3563,7 @@
         <v>4047</v>
       </c>
       <c r="K74" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B74, $C$2:$C$979, C74, $D$2:$D$979, D74, $E$2:$E$979, E74) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3572,23 +3571,23 @@
       <c r="A75" t="s">
         <v>61</v>
       </c>
-      <c r="B75" s="18" t="s">
+      <c r="B75" t="s">
         <v>62</v>
       </c>
-      <c r="C75" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D75" s="18">
+      <c r="C75" t="s">
+        <v>8</v>
+      </c>
+      <c r="D75">
         <v>2</v>
       </c>
-      <c r="E75" s="18">
+      <c r="E75">
         <v>4456</v>
       </c>
-      <c r="F75" s="18" t="s">
+      <c r="F75" t="s">
         <v>9</v>
       </c>
       <c r="G75">
-        <f>((E75-I75)/E75)*100</f>
+        <f t="shared" si="4"/>
         <v>-4.0260323159784477</v>
       </c>
       <c r="H75" s="9" t="s">
@@ -3598,7 +3597,7 @@
         <v>4635.3999999999996</v>
       </c>
       <c r="K75" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B75, $C$2:$C$979, C75, $D$2:$D$979, D75, $E$2:$E$979, E75) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3622,7 +3621,7 @@
         <v>9</v>
       </c>
       <c r="G76">
-        <f>((E76-I76)/E76)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.8709677419354889</v>
       </c>
       <c r="H76" s="9" t="s">
@@ -3632,31 +3631,31 @@
         <v>228.62</v>
       </c>
       <c r="K76" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B76, $C$2:$C$979, C76, $D$2:$D$979, D76, $E$2:$E$979, E76) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="77" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A77" s="18" t="s">
+      <c r="A77" t="s">
         <v>54</v>
       </c>
-      <c r="B77" s="18" t="s">
+      <c r="B77" t="s">
         <v>85</v>
       </c>
-      <c r="C77" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D77" s="18">
+      <c r="C77" t="s">
+        <v>8</v>
+      </c>
+      <c r="D77">
         <v>2</v>
       </c>
-      <c r="E77" s="18">
+      <c r="E77">
         <v>2460</v>
       </c>
-      <c r="F77" s="18" t="s">
+      <c r="F77" t="s">
         <v>9</v>
       </c>
       <c r="G77">
-        <f>((E77-I77)/E77)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.8699186991869845</v>
       </c>
       <c r="H77" s="9" t="s">
@@ -3666,7 +3665,7 @@
         <v>2555.1999999999998</v>
       </c>
       <c r="K77" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B77, $C$2:$C$979, C77, $D$2:$D$979, D77, $E$2:$E$979, E77) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3690,7 +3689,7 @@
         <v>9</v>
       </c>
       <c r="G78">
-        <f>((E78-I78)/E78)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.7878787878787881</v>
       </c>
       <c r="H78" s="9" t="s">
@@ -3700,7 +3699,7 @@
         <v>685</v>
       </c>
       <c r="K78" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B78, $C$2:$C$979, C78, $D$2:$D$979, D78, $E$2:$E$979, E78) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3724,7 +3723,7 @@
         <v>9</v>
       </c>
       <c r="G79">
-        <f>((E79-I79)/E79)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.7764705882352971</v>
       </c>
       <c r="H79" s="9" t="s">
@@ -3734,7 +3733,7 @@
         <v>882.1</v>
       </c>
       <c r="K79" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B79, $C$2:$C$979, C79, $D$2:$D$979, D79, $E$2:$E$979, E79) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3758,7 +3757,7 @@
         <v>9</v>
       </c>
       <c r="G80">
-        <f>((E80-I80)/E80)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.755868544600939</v>
       </c>
       <c r="H80" s="9" t="s">
@@ -3768,7 +3767,7 @@
         <v>442</v>
       </c>
       <c r="K80" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B80, $C$2:$C$979, C80, $D$2:$D$979, D80, $E$2:$E$979, E80) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3792,7 +3791,7 @@
         <v>9</v>
       </c>
       <c r="G81">
-        <f>((E81-I81)/E81)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.7068965517241317</v>
       </c>
       <c r="H81" s="9" t="s">
@@ -3802,7 +3801,7 @@
         <v>360.9</v>
       </c>
       <c r="K81" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B81, $C$2:$C$979, C81, $D$2:$D$979, D81, $E$2:$E$979, E81) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3826,7 +3825,7 @@
         <v>9</v>
       </c>
       <c r="G82">
-        <f>((E82-I82)/E82)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.5922330097087403</v>
       </c>
       <c r="H82" s="9" t="s">
@@ -3836,7 +3835,7 @@
         <v>213.4</v>
       </c>
       <c r="K82" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B82, $C$2:$C$979, C82, $D$2:$D$979, D82, $E$2:$E$979, E82) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3860,7 +3859,7 @@
         <v>9</v>
       </c>
       <c r="G83">
-        <f>((E83-I83)/E83)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.5315985130111525</v>
       </c>
       <c r="H83" s="9" t="s">
@@ -3870,7 +3869,7 @@
         <v>1671</v>
       </c>
       <c r="K83" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B83, $C$2:$C$979, C83, $D$2:$D$979, D83, $E$2:$E$979, E83) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3894,7 +3893,7 @@
         <v>9</v>
       </c>
       <c r="G84">
-        <f>((E84-I84)/E84)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.4623773173391492</v>
       </c>
       <c r="H84" s="9" t="s">
@@ -3904,7 +3903,7 @@
         <v>948.75</v>
       </c>
       <c r="K84" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B84, $C$2:$C$979, C84, $D$2:$D$979, D84, $E$2:$E$979, E84) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3928,7 +3927,7 @@
         <v>9</v>
       </c>
       <c r="G85">
-        <f>((E85-I85)/E85)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.2303370786516856</v>
       </c>
       <c r="H85" s="9" t="s">
@@ -3938,7 +3937,7 @@
         <v>735</v>
       </c>
       <c r="K85" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B85, $C$2:$C$979, C85, $D$2:$D$979, D85, $E$2:$E$979, E85) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3962,7 +3961,7 @@
         <v>9</v>
       </c>
       <c r="G86">
-        <f>((E86-I86)/E86)*100</f>
+        <f t="shared" si="4"/>
         <v>-3.1211498973305956</v>
       </c>
       <c r="H86" s="9" t="s">
@@ -3972,31 +3971,31 @@
         <v>2511</v>
       </c>
       <c r="K86" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B86, $C$2:$C$979, C86, $D$2:$D$979, D86, $E$2:$E$979, E86) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A87" s="18" t="s">
+      <c r="A87" t="s">
         <v>58</v>
       </c>
-      <c r="B87" s="18" t="s">
+      <c r="B87" t="s">
         <v>57</v>
       </c>
-      <c r="C87" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D87" s="18">
+      <c r="C87" t="s">
+        <v>8</v>
+      </c>
+      <c r="D87">
         <v>2</v>
       </c>
-      <c r="E87" s="18">
+      <c r="E87">
         <v>3410</v>
       </c>
-      <c r="F87" s="18" t="s">
+      <c r="F87" t="s">
         <v>9</v>
       </c>
       <c r="G87">
-        <f>((E87-I87)/E87)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.9618768328445748</v>
       </c>
       <c r="H87" s="9" t="s">
@@ -4006,31 +4005,31 @@
         <v>3511</v>
       </c>
       <c r="K87" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B87, $C$2:$C$979, C87, $D$2:$D$979, D87, $E$2:$E$979, E87) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A88" s="18" t="s">
+      <c r="A88" t="s">
         <v>73</v>
       </c>
-      <c r="B88" s="18" t="s">
+      <c r="B88" t="s">
         <v>83</v>
       </c>
-      <c r="C88" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D88" s="18">
+      <c r="C88" t="s">
+        <v>8</v>
+      </c>
+      <c r="D88">
         <v>1</v>
       </c>
-      <c r="E88" s="18">
+      <c r="E88">
         <v>4306</v>
       </c>
-      <c r="F88" s="18" t="s">
+      <c r="F88" t="s">
         <v>9</v>
       </c>
       <c r="G88">
-        <f>((E88-I88)/E88)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.9168601950766457</v>
       </c>
       <c r="H88" s="9" t="s">
@@ -4040,31 +4039,31 @@
         <v>4431.6000000000004</v>
       </c>
       <c r="K88" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B88, $C$2:$C$979, C88, $D$2:$D$979, D88, $E$2:$E$979, E88) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A89" s="18" t="s">
+      <c r="A89" t="s">
         <v>73</v>
       </c>
-      <c r="B89" s="18" t="s">
+      <c r="B89" t="s">
         <v>95</v>
       </c>
-      <c r="C89" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D89" s="18">
+      <c r="C89" t="s">
+        <v>8</v>
+      </c>
+      <c r="D89">
         <v>5</v>
       </c>
-      <c r="E89" s="18">
+      <c r="E89">
         <v>3938</v>
       </c>
-      <c r="F89" s="18" t="s">
+      <c r="F89" t="s">
         <v>9</v>
       </c>
       <c r="G89">
-        <f>((E89-I89)/E89)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.7679024885728798</v>
       </c>
       <c r="H89" s="9" t="s">
@@ -4074,7 +4073,7 @@
         <v>4047</v>
       </c>
       <c r="K89" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B89, $C$2:$C$979, C89, $D$2:$D$979, D89, $E$2:$E$979, E89) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4098,7 +4097,7 @@
         <v>9</v>
       </c>
       <c r="G90">
-        <f>((E90-I90)/E90)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.6562500000000044</v>
       </c>
       <c r="H90" s="9" t="s">
@@ -4108,7 +4107,7 @@
         <v>131.4</v>
       </c>
       <c r="K90" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B90, $C$2:$C$979, C90, $D$2:$D$979, D90, $E$2:$E$979, E90) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4132,7 +4131,7 @@
         <v>9</v>
       </c>
       <c r="G91">
-        <f>((E91-I91)/E91)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.6445578231292441</v>
       </c>
       <c r="H91" s="9" t="s">
@@ -4142,7 +4141,7 @@
         <v>2414.1999999999998</v>
       </c>
       <c r="K91" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B91, $C$2:$C$979, C91, $D$2:$D$979, D91, $E$2:$E$979, E91) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4166,7 +4165,7 @@
         <v>9</v>
       </c>
       <c r="G92">
-        <f>((E92-I92)/E92)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.5284090909090842</v>
       </c>
       <c r="H92" s="9" t="s">
@@ -4176,31 +4175,31 @@
         <v>360.9</v>
       </c>
       <c r="K92" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B92, $C$2:$C$979, C92, $D$2:$D$979, D92, $E$2:$E$979, E92) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A93" s="18" t="s">
+      <c r="A93" t="s">
         <v>96</v>
       </c>
-      <c r="B93" s="18" t="s">
+      <c r="B93" t="s">
         <v>95</v>
       </c>
-      <c r="C93" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D93" s="18">
+      <c r="C93" t="s">
+        <v>8</v>
+      </c>
+      <c r="D93">
         <v>10</v>
       </c>
-      <c r="E93" s="18">
+      <c r="E93">
         <v>3950</v>
       </c>
-      <c r="F93" s="18" t="s">
+      <c r="F93" t="s">
         <v>9</v>
       </c>
       <c r="G93">
-        <f>((E93-I93)/E93)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.4556962025316453</v>
       </c>
       <c r="H93" s="9" t="s">
@@ -4210,7 +4209,7 @@
         <v>4047</v>
       </c>
       <c r="K93" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B93, $C$2:$C$979, C93, $D$2:$D$979, D93, $E$2:$E$979, E93) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4234,7 +4233,7 @@
         <v>9</v>
       </c>
       <c r="G94">
-        <f>((E94-I94)/E94)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.3770491803278717</v>
       </c>
       <c r="H94" s="9" t="s">
@@ -4244,7 +4243,7 @@
         <v>811.85</v>
       </c>
       <c r="K94" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B94, $C$2:$C$979, C94, $D$2:$D$979, D94, $E$2:$E$979, E94) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4268,7 +4267,7 @@
         <v>9</v>
       </c>
       <c r="G95">
-        <f>((E95-I95)/E95)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.3462783171521036</v>
       </c>
       <c r="H95" s="9" t="s">
@@ -4278,7 +4277,7 @@
         <v>948.75</v>
       </c>
       <c r="K95" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B95, $C$2:$C$979, C95, $D$2:$D$979, D95, $E$2:$E$979, E95) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4302,7 +4301,7 @@
         <v>9</v>
       </c>
       <c r="G96">
-        <f>((E96-I96)/E96)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.1505376344086025</v>
       </c>
       <c r="H96" s="9" t="s">
@@ -4312,7 +4311,7 @@
         <v>1330</v>
       </c>
       <c r="K96" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B96, $C$2:$C$979, C96, $D$2:$D$979, D96, $E$2:$E$979, E96) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4336,7 +4335,7 @@
         <v>9</v>
       </c>
       <c r="G97">
-        <f>((E97-I97)/E97)*100</f>
+        <f t="shared" si="4"/>
         <v>-2.0731707317073171</v>
       </c>
       <c r="H97" s="9" t="s">
@@ -4346,7 +4345,7 @@
         <v>2511</v>
       </c>
       <c r="K97" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B97, $C$2:$C$979, C97, $D$2:$D$979, D97, $E$2:$E$979, E97) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4370,7 +4369,7 @@
         <v>9</v>
       </c>
       <c r="G98">
-        <f>((E98-I98)/E98)*100</f>
+        <f t="shared" ref="G98:G129" si="6">((E98-I98)/E98)*100</f>
         <v>-1.8221003134796239</v>
       </c>
       <c r="H98" s="9" t="s">
@@ -4380,7 +4379,7 @@
         <v>2598.5</v>
       </c>
       <c r="K98" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B98, $C$2:$C$979, C98, $D$2:$D$979, D98, $E$2:$E$979, E98) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="K98:K129" si="7">IF(COUNTIFS( $B$2:$B$979, B98, $C$2:$C$979, C98, $D$2:$D$979, D98, $E$2:$E$979, E98) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -4404,7 +4403,7 @@
         <v>9</v>
       </c>
       <c r="G99">
-        <f>((E99-I99)/E99)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.8098510882016017</v>
       </c>
       <c r="H99" s="9" t="s">
@@ -4414,31 +4413,31 @@
         <v>88.88</v>
       </c>
       <c r="K99" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B99, $C$2:$C$979, C99, $D$2:$D$979, D99, $E$2:$E$979, E99) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A100" s="18" t="s">
+      <c r="A100" t="s">
         <v>73</v>
       </c>
-      <c r="B100" s="18" t="s">
+      <c r="B100" t="s">
         <v>62</v>
       </c>
-      <c r="C100" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D100" s="18">
+      <c r="C100" t="s">
+        <v>8</v>
+      </c>
+      <c r="D100">
         <v>1</v>
       </c>
-      <c r="E100" s="18">
+      <c r="E100">
         <v>4560</v>
       </c>
-      <c r="F100" s="18" t="s">
+      <c r="F100" t="s">
         <v>9</v>
       </c>
       <c r="G100">
-        <f>((E100-I100)/E100)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.6535087719298167</v>
       </c>
       <c r="H100" s="9" t="s">
@@ -4448,31 +4447,31 @@
         <v>4635.3999999999996</v>
       </c>
       <c r="K100" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B100, $C$2:$C$979, C100, $D$2:$D$979, D100, $E$2:$E$979, E100) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A101" s="18" t="s">
+      <c r="A101" t="s">
         <v>58</v>
       </c>
-      <c r="B101" s="18" t="s">
+      <c r="B101" t="s">
         <v>81</v>
       </c>
-      <c r="C101" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D101" s="18">
+      <c r="C101" t="s">
+        <v>8</v>
+      </c>
+      <c r="D101">
         <v>2</v>
       </c>
-      <c r="E101" s="18">
+      <c r="E101">
         <v>2560</v>
       </c>
-      <c r="F101" s="18" t="s">
+      <c r="F101" t="s">
         <v>9</v>
       </c>
       <c r="G101">
-        <f>((E101-I101)/E101)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.50390625</v>
       </c>
       <c r="H101" s="9" t="s">
@@ -4482,7 +4481,7 @@
         <v>2598.5</v>
       </c>
       <c r="K101" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B101, $C$2:$C$979, C101, $D$2:$D$979, D101, $E$2:$E$979, E101) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4506,7 +4505,7 @@
         <v>9</v>
       </c>
       <c r="G102">
-        <f>((E102-I102)/E102)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.4189189189189151</v>
       </c>
       <c r="H102" s="9" t="s">
@@ -4516,7 +4515,7 @@
         <v>300.2</v>
       </c>
       <c r="K102" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B102, $C$2:$C$979, C102, $D$2:$D$979, D102, $E$2:$E$979, E102) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4540,7 +4539,7 @@
         <v>9</v>
       </c>
       <c r="G103">
-        <f>((E103-I103)/E103)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.4150943396226416</v>
       </c>
       <c r="H103" s="9" t="s">
@@ -4550,7 +4549,7 @@
         <v>1075</v>
       </c>
       <c r="K103" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B103, $C$2:$C$979, C103, $D$2:$D$979, D103, $E$2:$E$979, E103) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4574,7 +4573,7 @@
         <v>9</v>
       </c>
       <c r="G104">
-        <f>((E104-I104)/E104)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.3761467889908259</v>
       </c>
       <c r="H104" s="9" t="s">
@@ -4584,7 +4583,7 @@
         <v>442</v>
       </c>
       <c r="K104" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B104, $C$2:$C$979, C104, $D$2:$D$979, D104, $E$2:$E$979, E104) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4608,7 +4607,7 @@
         <v>9</v>
       </c>
       <c r="G105">
-        <f>((E105-I105)/E105)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.2396694214876034</v>
       </c>
       <c r="H105" s="9" t="s">
@@ -4618,7 +4617,7 @@
         <v>735</v>
       </c>
       <c r="K105" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B105, $C$2:$C$979, C105, $D$2:$D$979, D105, $E$2:$E$979, E105) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4642,7 +4641,7 @@
         <v>9</v>
       </c>
       <c r="G106">
-        <f>((E106-I106)/E106)*100</f>
+        <f t="shared" si="6"/>
         <v>-1.2237762237762237</v>
       </c>
       <c r="H106" s="9" t="s">
@@ -4652,7 +4651,7 @@
         <v>289.5</v>
       </c>
       <c r="K106" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B106, $C$2:$C$979, C106, $D$2:$D$979, D106, $E$2:$E$979, E106) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4676,7 +4675,7 @@
         <v>9</v>
       </c>
       <c r="G107">
-        <f>((E107-I107)/E107)*100</f>
+        <f t="shared" si="6"/>
         <v>-0.70921985815602839</v>
       </c>
       <c r="H107" s="9" t="s">
@@ -4686,7 +4685,7 @@
         <v>1420</v>
       </c>
       <c r="K107" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B107, $C$2:$C$979, C107, $D$2:$D$979, D107, $E$2:$E$979, E107) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4710,7 +4709,7 @@
         <v>9</v>
       </c>
       <c r="G108">
-        <f>((E108-I108)/E108)*100</f>
+        <f t="shared" si="6"/>
         <v>-0.49230769230769433</v>
       </c>
       <c r="H108" s="9" t="s">
@@ -4720,7 +4719,7 @@
         <v>228.62</v>
       </c>
       <c r="K108" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B108, $C$2:$C$979, C108, $D$2:$D$979, D108, $E$2:$E$979, E108) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4744,7 +4743,7 @@
         <v>9</v>
       </c>
       <c r="G109">
-        <f>((E109-I109)/E109)*100</f>
+        <f t="shared" si="6"/>
         <v>0.14204545454545456</v>
       </c>
       <c r="H109" s="9" t="s">
@@ -4754,7 +4753,7 @@
         <v>1054.5</v>
       </c>
       <c r="K109" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B109, $C$2:$C$979, C109, $D$2:$D$979, D109, $E$2:$E$979, E109) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4778,7 +4777,7 @@
         <v>9</v>
       </c>
       <c r="G110">
-        <f>((E110-I110)/E110)*100</f>
+        <f t="shared" si="6"/>
         <v>0.77805077805077805</v>
       </c>
       <c r="H110" s="9" t="s">
@@ -4788,7 +4787,7 @@
         <v>1211.5</v>
       </c>
       <c r="K110" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B110, $C$2:$C$979, C110, $D$2:$D$979, D110, $E$2:$E$979, E110) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4812,7 +4811,7 @@
         <v>9</v>
       </c>
       <c r="G111">
-        <f>((E111-I111)/E111)*100</f>
+        <f t="shared" si="6"/>
         <v>1.5513392857142831</v>
       </c>
       <c r="H111" s="9" t="s">
@@ -4822,7 +4821,7 @@
         <v>882.1</v>
       </c>
       <c r="K111" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B111, $C$2:$C$979, C111, $D$2:$D$979, D111, $E$2:$E$979, E111) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4846,7 +4845,7 @@
         <v>9</v>
       </c>
       <c r="G112">
-        <f>((E112-I112)/E112)*100</f>
+        <f t="shared" si="6"/>
         <v>1.6204941704995188</v>
       </c>
       <c r="H112" s="9" t="s">
@@ -4856,31 +4855,31 @@
         <v>18395</v>
       </c>
       <c r="K112" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B112, $C$2:$C$979, C112, $D$2:$D$979, D112, $E$2:$E$979, E112) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A113" s="18" t="s">
+      <c r="A113" t="s">
         <v>66</v>
       </c>
-      <c r="B113" s="18" t="s">
+      <c r="B113" t="s">
         <v>95</v>
       </c>
-      <c r="C113" s="18" t="s">
+      <c r="C113" t="s">
         <v>14</v>
       </c>
-      <c r="D113" s="18">
+      <c r="D113">
         <v>5</v>
       </c>
-      <c r="E113" s="18">
+      <c r="E113">
         <v>4129</v>
       </c>
-      <c r="F113" s="18" t="s">
+      <c r="F113" t="s">
         <v>9</v>
       </c>
       <c r="G113">
-        <f>((E113-I113)/E113)*100</f>
+        <f t="shared" si="6"/>
         <v>1.9859530152579317</v>
       </c>
       <c r="H113" s="9" t="s">
@@ -4890,7 +4889,7 @@
         <v>4047</v>
       </c>
       <c r="K113" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B113, $C$2:$C$979, C113, $D$2:$D$979, D113, $E$2:$E$979, E113) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4914,7 +4913,7 @@
         <v>9</v>
       </c>
       <c r="G114">
-        <f>((E114-I114)/E114)*100</f>
+        <f t="shared" si="6"/>
         <v>2.0606060606060654</v>
       </c>
       <c r="H114" s="9" t="s">
@@ -4924,7 +4923,7 @@
         <v>88.88</v>
       </c>
       <c r="K114" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B114, $C$2:$C$979, C114, $D$2:$D$979, D114, $E$2:$E$979, E114) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4948,7 +4947,7 @@
         <v>9</v>
       </c>
       <c r="G115">
-        <f>((E115-I115)/E115)*100</f>
+        <f t="shared" si="6"/>
         <v>2.1069692058346909</v>
       </c>
       <c r="H115" s="9" t="s">
@@ -4958,7 +4957,7 @@
         <v>120.8</v>
       </c>
       <c r="K115" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B115, $C$2:$C$979, C115, $D$2:$D$979, D115, $E$2:$E$979, E115) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4982,7 +4981,7 @@
         <v>9</v>
       </c>
       <c r="G116">
-        <f>((E116-I116)/E116)*100</f>
+        <f t="shared" si="6"/>
         <v>2.1100917431192636</v>
       </c>
       <c r="H116" s="9" t="s">
@@ -4992,7 +4991,7 @@
         <v>213.4</v>
       </c>
       <c r="K116" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B116, $C$2:$C$979, C116, $D$2:$D$979, D116, $E$2:$E$979, E116) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5016,7 +5015,7 @@
         <v>9</v>
       </c>
       <c r="G117">
-        <f>((E117-I117)/E117)*100</f>
+        <f t="shared" si="6"/>
         <v>2.2991452991452972</v>
       </c>
       <c r="H117" s="9" t="s">
@@ -5026,7 +5025,7 @@
         <v>228.62</v>
       </c>
       <c r="K117" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B117, $C$2:$C$979, C117, $D$2:$D$979, D117, $E$2:$E$979, E117) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5050,7 +5049,7 @@
         <v>9</v>
       </c>
       <c r="G118">
-        <f>((E118-I118)/E118)*100</f>
+        <f t="shared" si="6"/>
         <v>2.5222551928783425</v>
       </c>
       <c r="H118" s="9" t="s">
@@ -5060,7 +5059,7 @@
         <v>131.4</v>
       </c>
       <c r="K118" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B118, $C$2:$C$979, C118, $D$2:$D$979, D118, $E$2:$E$979, E118) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5084,7 +5083,7 @@
         <v>9</v>
       </c>
       <c r="G119">
-        <f>((E119-I119)/E119)*100</f>
+        <f t="shared" si="6"/>
         <v>2.6214953271028101</v>
       </c>
       <c r="H119" s="9" t="s">
@@ -5094,7 +5093,7 @@
         <v>208.39</v>
       </c>
       <c r="K119" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B119, $C$2:$C$979, C119, $D$2:$D$979, D119, $E$2:$E$979, E119) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5118,7 +5117,7 @@
         <v>9</v>
       </c>
       <c r="G120">
-        <f>((E120-I120)/E120)*100</f>
+        <f t="shared" si="6"/>
         <v>2.622950819672131</v>
       </c>
       <c r="H120" s="9" t="s">
@@ -5128,7 +5127,7 @@
         <v>2376</v>
       </c>
       <c r="K120" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B120, $C$2:$C$979, C120, $D$2:$D$979, D120, $E$2:$E$979, E120) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5152,7 +5151,7 @@
         <v>9</v>
       </c>
       <c r="G121">
-        <f>((E121-I121)/E121)*100</f>
+        <f t="shared" si="6"/>
         <v>2.7397260273972601</v>
       </c>
       <c r="H121" s="9" t="s">
@@ -5162,7 +5161,7 @@
         <v>1420</v>
       </c>
       <c r="K121" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B121, $C$2:$C$979, C121, $D$2:$D$979, D121, $E$2:$E$979, E121) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5186,7 +5185,7 @@
         <v>9</v>
       </c>
       <c r="G122">
-        <f>((E122-I122)/E122)*100</f>
+        <f t="shared" si="6"/>
         <v>2.8915046059365404</v>
       </c>
       <c r="H122" s="9" t="s">
@@ -5196,12 +5195,12 @@
         <v>948.75</v>
       </c>
       <c r="K122" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B122, $C$2:$C$979, C122, $D$2:$D$979, D122, $E$2:$E$979, E122) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A123" s="19">
+      <c r="A123" s="18">
         <v>46239</v>
       </c>
       <c r="B123" s="15" t="s">
@@ -5220,7 +5219,7 @@
         <v>9</v>
       </c>
       <c r="G123">
-        <f>((E123-I123)/E123)*100</f>
+        <f t="shared" si="6"/>
         <v>3.0501930501930499</v>
       </c>
       <c r="H123" s="9" t="s">
@@ -5230,7 +5229,7 @@
         <v>2511</v>
       </c>
       <c r="K123" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B123, $C$2:$C$979, C123, $D$2:$D$979, D123, $E$2:$E$979, E123) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5254,7 +5253,7 @@
         <v>9</v>
       </c>
       <c r="G124">
-        <f>((E124-I124)/E124)*100</f>
+        <f t="shared" si="6"/>
         <v>3.1122815417763947</v>
       </c>
       <c r="H124" s="9" t="s">
@@ -5264,7 +5263,7 @@
         <v>4047</v>
       </c>
       <c r="K124" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B124, $C$2:$C$979, C124, $D$2:$D$979, D124, $E$2:$E$979, E124) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5288,7 +5287,7 @@
         <v>9</v>
       </c>
       <c r="G125">
-        <f>((E125-I125)/E125)*100</f>
+        <f t="shared" si="6"/>
         <v>3.1280653950953732</v>
       </c>
       <c r="H125" s="9" t="s">
@@ -5298,7 +5297,7 @@
         <v>88.88</v>
       </c>
       <c r="K125" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B125, $C$2:$C$979, C125, $D$2:$D$979, D125, $E$2:$E$979, E125) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5322,7 +5321,7 @@
         <v>9</v>
       </c>
       <c r="G126">
-        <f>((E126-I126)/E126)*100</f>
+        <f t="shared" si="6"/>
         <v>3.2031249999999996</v>
       </c>
       <c r="H126" s="9" t="s">
@@ -5332,7 +5331,7 @@
         <v>1239</v>
       </c>
       <c r="K126" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B126, $C$2:$C$979, C126, $D$2:$D$979, D126, $E$2:$E$979, E126) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5356,7 +5355,7 @@
         <v>9</v>
       </c>
       <c r="G127">
-        <f>((E127-I127)/E127)*100</f>
+        <f t="shared" si="6"/>
         <v>3.2439678284182363</v>
       </c>
       <c r="H127" s="9" t="s">
@@ -5366,7 +5365,7 @@
         <v>360.9</v>
       </c>
       <c r="K127" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B127, $C$2:$C$979, C127, $D$2:$D$979, D127, $E$2:$E$979, E127) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5390,7 +5389,7 @@
         <v>9</v>
       </c>
       <c r="G128">
-        <f>((E128-I128)/E128)*100</f>
+        <f t="shared" si="6"/>
         <v>3.2826261008807109</v>
       </c>
       <c r="H128" s="9" t="s">
@@ -5400,31 +5399,31 @@
         <v>120.8</v>
       </c>
       <c r="K128" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B128, $C$2:$C$979, C128, $D$2:$D$979, D128, $E$2:$E$979, E128) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A129" s="18" t="s">
+      <c r="A129" t="s">
         <v>56</v>
       </c>
-      <c r="B129" s="18" t="s">
+      <c r="B129" t="s">
         <v>57</v>
       </c>
-      <c r="C129" s="18" t="s">
+      <c r="C129" t="s">
         <v>14</v>
       </c>
-      <c r="D129" s="18">
+      <c r="D129">
         <v>5</v>
       </c>
-      <c r="E129" s="18">
+      <c r="E129">
         <v>3633</v>
       </c>
-      <c r="F129" s="18" t="s">
+      <c r="F129" t="s">
         <v>9</v>
       </c>
       <c r="G129">
-        <f>((E129-I129)/E129)*100</f>
+        <f t="shared" si="6"/>
         <v>3.3581062482796589</v>
       </c>
       <c r="H129" s="9" t="s">
@@ -5434,7 +5433,7 @@
         <v>3511</v>
       </c>
       <c r="K129" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B129, $C$2:$C$979, C129, $D$2:$D$979, D129, $E$2:$E$979, E129) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5458,7 +5457,7 @@
         <v>9</v>
       </c>
       <c r="G130">
-        <f>((E130-I130)/E130)*100</f>
+        <f t="shared" ref="G130:G161" si="8">((E130-I130)/E130)*100</f>
         <v>3.3823529411764661</v>
       </c>
       <c r="H130" s="9" t="s">
@@ -5468,31 +5467,31 @@
         <v>131.4</v>
       </c>
       <c r="K130" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B130, $C$2:$C$979, C130, $D$2:$D$979, D130, $E$2:$E$979, E130) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="K130:K161" si="9">IF(COUNTIFS( $B$2:$B$979, B130, $C$2:$C$979, C130, $D$2:$D$979, D130, $E$2:$E$979, E130) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A131" s="18" t="s">
+      <c r="A131" t="s">
         <v>74</v>
       </c>
-      <c r="B131" s="18" t="s">
+      <c r="B131" t="s">
         <v>75</v>
       </c>
-      <c r="C131" s="18" t="s">
+      <c r="C131" t="s">
         <v>14</v>
       </c>
-      <c r="D131" s="18">
+      <c r="D131">
         <v>5</v>
       </c>
-      <c r="E131" s="18">
+      <c r="E131">
         <v>4040</v>
       </c>
-      <c r="F131" s="18" t="s">
+      <c r="F131" t="s">
         <v>9</v>
       </c>
       <c r="G131">
-        <f>((E131-I131)/E131)*100</f>
+        <f t="shared" si="8"/>
         <v>3.5148514851485153</v>
       </c>
       <c r="H131" s="9" t="s">
@@ -5502,7 +5501,7 @@
         <v>3898</v>
       </c>
       <c r="K131" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B131, $C$2:$C$979, C131, $D$2:$D$979, D131, $E$2:$E$979, E131) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5526,7 +5525,7 @@
         <v>9</v>
       </c>
       <c r="G132">
-        <f>((E132-I132)/E132)*100</f>
+        <f t="shared" si="8"/>
         <v>3.6605657237936775</v>
       </c>
       <c r="H132" s="9" t="s">
@@ -5536,7 +5535,7 @@
         <v>289.5</v>
       </c>
       <c r="K132" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B132, $C$2:$C$979, C132, $D$2:$D$979, D132, $E$2:$E$979, E132) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5560,7 +5559,7 @@
         <v>9</v>
       </c>
       <c r="G133">
-        <f>((E133-I133)/E133)*100</f>
+        <f t="shared" si="8"/>
         <v>3.8095238095238098</v>
       </c>
       <c r="H133" s="9" t="s">
@@ -5570,7 +5569,7 @@
         <v>202</v>
       </c>
       <c r="K133" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B133, $C$2:$C$979, C133, $D$2:$D$979, D133, $E$2:$E$979, E133) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5594,7 +5593,7 @@
         <v>9</v>
       </c>
       <c r="G134">
-        <f>((E134-I134)/E134)*100</f>
+        <f t="shared" si="8"/>
         <v>3.8518518518518579</v>
       </c>
       <c r="H134" s="9" t="s">
@@ -5604,7 +5603,7 @@
         <v>389.4</v>
       </c>
       <c r="K134" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B134, $C$2:$C$979, C134, $D$2:$D$979, D134, $E$2:$E$979, E134) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5628,7 +5627,7 @@
         <v>9</v>
       </c>
       <c r="G135">
-        <f>((E135-I135)/E135)*100</f>
+        <f t="shared" si="8"/>
         <v>4.0218303946263578</v>
       </c>
       <c r="H135" s="9" t="s">
@@ -5638,7 +5637,7 @@
         <v>228.62</v>
       </c>
       <c r="K135" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B135, $C$2:$C$979, C135, $D$2:$D$979, D135, $E$2:$E$979, E135) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5662,7 +5661,7 @@
         <v>9</v>
       </c>
       <c r="G136">
-        <f>((E136-I136)/E136)*100</f>
+        <f t="shared" si="8"/>
         <v>4.0870893812070284</v>
       </c>
       <c r="H136" s="9" t="s">
@@ -5673,7 +5672,7 @@
       </c>
       <c r="J136"/>
       <c r="K136" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B136, $C$2:$C$979, C136, $D$2:$D$979, D136, $E$2:$E$979, E136) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5697,7 +5696,7 @@
         <v>9</v>
       </c>
       <c r="G137">
-        <f>((E137-I137)/E137)*100</f>
+        <f t="shared" si="8"/>
         <v>4.1603053435114496</v>
       </c>
       <c r="H137" s="9" t="s">
@@ -5707,7 +5706,7 @@
         <v>2511</v>
       </c>
       <c r="K137" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B137, $C$2:$C$979, C137, $D$2:$D$979, D137, $E$2:$E$979, E137) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5731,7 +5730,7 @@
         <v>9</v>
       </c>
       <c r="G138">
-        <f>((E138-I138)/E138)*100</f>
+        <f t="shared" si="8"/>
         <v>4.1725067385444792</v>
       </c>
       <c r="H138" s="9" t="s">
@@ -5741,7 +5740,7 @@
         <v>88.88</v>
       </c>
       <c r="K138" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B138, $C$2:$C$979, C138, $D$2:$D$979, D138, $E$2:$E$979, E138) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5765,7 +5764,7 @@
         <v>9</v>
       </c>
       <c r="G139">
-        <f>((E139-I139)/E139)*100</f>
+        <f t="shared" si="8"/>
         <v>4.182727367434107</v>
       </c>
       <c r="H139" s="9" t="s">
@@ -5775,7 +5774,7 @@
         <v>18395</v>
       </c>
       <c r="K139" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B139, $C$2:$C$979, C139, $D$2:$D$979, D139, $E$2:$E$979, E139) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5799,7 +5798,7 @@
         <v>9</v>
       </c>
       <c r="G140">
-        <f>((E140-I140)/E140)*100</f>
+        <f t="shared" si="8"/>
         <v>4.3430962343096216</v>
       </c>
       <c r="H140" s="9" t="s">
@@ -5809,7 +5808,7 @@
         <v>228.62</v>
       </c>
       <c r="K140" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B140, $C$2:$C$979, C140, $D$2:$D$979, D140, $E$2:$E$979, E140) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5833,7 +5832,7 @@
         <v>9</v>
       </c>
       <c r="G141">
-        <f>((E141-I141)/E141)*100</f>
+        <f t="shared" si="8"/>
         <v>4.5358649789029535</v>
       </c>
       <c r="H141" s="9" t="s">
@@ -5843,7 +5842,7 @@
         <v>905</v>
       </c>
       <c r="K141" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B141, $C$2:$C$979, C141, $D$2:$D$979, D141, $E$2:$E$979, E141) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5867,7 +5866,7 @@
         <v>9</v>
       </c>
       <c r="G142">
-        <f>((E142-I142)/E142)*100</f>
+        <f t="shared" si="8"/>
         <v>4.5454545454545459</v>
       </c>
       <c r="H142" s="9" t="s">
@@ -5877,7 +5876,7 @@
         <v>1239</v>
       </c>
       <c r="K142" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B142, $C$2:$C$979, C142, $D$2:$D$979, D142, $E$2:$E$979, E142) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5901,7 +5900,7 @@
         <v>9</v>
       </c>
       <c r="G143">
-        <f>((E143-I143)/E143)*100</f>
+        <f t="shared" si="8"/>
         <v>4.5783132530120483</v>
       </c>
       <c r="H143" s="9" t="s">
@@ -5911,7 +5910,7 @@
         <v>2376</v>
       </c>
       <c r="K143" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B143, $C$2:$C$979, C143, $D$2:$D$979, D143, $E$2:$E$979, E143) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5935,7 +5934,7 @@
         <v>9</v>
       </c>
       <c r="G144">
-        <f>((E144-I144)/E144)*100</f>
+        <f t="shared" si="8"/>
         <v>4.6979865771812079</v>
       </c>
       <c r="H144" s="9" t="s">
@@ -5945,7 +5944,7 @@
         <v>1420</v>
       </c>
       <c r="K144" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B144, $C$2:$C$979, C144, $D$2:$D$979, D144, $E$2:$E$979, E144) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5969,7 +5968,7 @@
         <v>9</v>
       </c>
       <c r="G145">
-        <f>((E145-I145)/E145)*100</f>
+        <f t="shared" si="8"/>
         <v>4.8395185556670013</v>
       </c>
       <c r="H145" s="9" t="s">
@@ -5979,7 +5978,7 @@
         <v>948.75</v>
       </c>
       <c r="K145" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B145, $C$2:$C$979, C145, $D$2:$D$979, D145, $E$2:$E$979, E145) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6003,7 +6002,7 @@
         <v>9</v>
       </c>
       <c r="G146">
-        <f>((E146-I146)/E146)*100</f>
+        <f t="shared" si="8"/>
         <v>4.8447488584474954</v>
       </c>
       <c r="H146" s="9" t="s">
@@ -6013,7 +6012,7 @@
         <v>208.39</v>
       </c>
       <c r="K146" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B146, $C$2:$C$979, C146, $D$2:$D$979, D146, $E$2:$E$979, E146) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6037,7 +6036,7 @@
         <v>9</v>
       </c>
       <c r="G147">
-        <f>((E147-I147)/E147)*100</f>
+        <f t="shared" si="8"/>
         <v>5.0111524163568841</v>
       </c>
       <c r="H147" s="9" t="s">
@@ -6047,7 +6046,7 @@
         <v>2555.1999999999998</v>
       </c>
       <c r="K147" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B147, $C$2:$C$979, C147, $D$2:$D$979, D147, $E$2:$E$979, E147) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6071,7 +6070,7 @@
         <v>9</v>
       </c>
       <c r="G148">
-        <f>((E148-I148)/E148)*100</f>
+        <f t="shared" si="8"/>
         <v>5.1737160120845918</v>
       </c>
       <c r="H148" s="9" t="s">
@@ -6081,7 +6080,7 @@
         <v>2511</v>
       </c>
       <c r="K148" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B148, $C$2:$C$979, C148, $D$2:$D$979, D148, $E$2:$E$979, E148) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6105,7 +6104,7 @@
         <v>9</v>
       </c>
       <c r="G149">
-        <f>((E149-I149)/E149)*100</f>
+        <f t="shared" si="8"/>
         <v>5.2065439672801705</v>
       </c>
       <c r="H149" s="9" t="s">
@@ -6115,7 +6114,7 @@
         <v>4635.3999999999996</v>
       </c>
       <c r="K149" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B149, $C$2:$C$979, C149, $D$2:$D$979, D149, $E$2:$E$979, E149) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6139,7 +6138,7 @@
         <v>9</v>
       </c>
       <c r="G150">
-        <f>((E150-I150)/E150)*100</f>
+        <f t="shared" si="8"/>
         <v>5.2919708029197077</v>
       </c>
       <c r="H150" s="9" t="s">
@@ -6149,7 +6148,7 @@
         <v>519</v>
       </c>
       <c r="K150" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B150, $C$2:$C$979, C150, $D$2:$D$979, D150, $E$2:$E$979, E150) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6173,7 +6172,7 @@
         <v>9</v>
       </c>
       <c r="G151">
-        <f>((E151-I151)/E151)*100</f>
+        <f t="shared" si="8"/>
         <v>5.3638814016172507</v>
       </c>
       <c r="H151" s="9" t="s">
@@ -6183,7 +6182,7 @@
         <v>3511</v>
       </c>
       <c r="K151" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B151, $C$2:$C$979, C151, $D$2:$D$979, D151, $E$2:$E$979, E151) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6207,7 +6206,7 @@
         <v>9</v>
       </c>
       <c r="G152">
-        <f>((E152-I152)/E152)*100</f>
+        <f t="shared" si="8"/>
         <v>5.4039593365436058</v>
       </c>
       <c r="H152" s="9" t="s">
@@ -6217,7 +6216,7 @@
         <v>442</v>
       </c>
       <c r="K152" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B152, $C$2:$C$979, C152, $D$2:$D$979, D152, $E$2:$E$979, E152) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6241,7 +6240,7 @@
         <v>9</v>
       </c>
       <c r="G153">
-        <f>((E153-I153)/E153)*100</f>
+        <f t="shared" si="8"/>
         <v>5.6074766355140184</v>
       </c>
       <c r="H153" s="9" t="s">
@@ -6251,7 +6250,7 @@
         <v>202</v>
       </c>
       <c r="K153" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B153, $C$2:$C$979, C153, $D$2:$D$979, D153, $E$2:$E$979, E153) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6275,7 +6274,7 @@
         <v>9</v>
       </c>
       <c r="G154">
-        <f>((E154-I154)/E154)*100</f>
+        <f t="shared" si="8"/>
         <v>5.7121771217712247</v>
       </c>
       <c r="H154" s="9" t="s">
@@ -6285,7 +6284,7 @@
         <v>2555.1999999999998</v>
       </c>
       <c r="K154" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B154, $C$2:$C$979, C154, $D$2:$D$979, D154, $E$2:$E$979, E154) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6309,7 +6308,7 @@
         <v>9</v>
       </c>
       <c r="G155">
-        <f>((E155-I155)/E155)*100</f>
+        <f t="shared" si="8"/>
         <v>6.0254491017964078</v>
       </c>
       <c r="H155" s="9" t="s">
@@ -6319,7 +6318,7 @@
         <v>2511</v>
       </c>
       <c r="K155" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B155, $C$2:$C$979, C155, $D$2:$D$979, D155, $E$2:$E$979, E155) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6343,7 +6342,7 @@
         <v>9</v>
       </c>
       <c r="G156">
-        <f>((E156-I156)/E156)*100</f>
+        <f t="shared" si="8"/>
         <v>6.1643835616438354</v>
       </c>
       <c r="H156" s="9" t="s">
@@ -6353,7 +6352,7 @@
         <v>685</v>
       </c>
       <c r="K156" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B156, $C$2:$C$979, C156, $D$2:$D$979, D156, $E$2:$E$979, E156) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6377,7 +6376,7 @@
         <v>9</v>
       </c>
       <c r="G157">
-        <f>((E157-I157)/E157)*100</f>
+        <f t="shared" si="8"/>
         <v>6.3032786885245882</v>
       </c>
       <c r="H157" s="9" t="s">
@@ -6387,7 +6386,7 @@
         <v>228.62</v>
       </c>
       <c r="K157" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B157, $C$2:$C$979, C157, $D$2:$D$979, D157, $E$2:$E$979, E157) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6411,7 +6410,7 @@
         <v>9</v>
       </c>
       <c r="G158">
-        <f>((E158-I158)/E158)*100</f>
+        <f t="shared" si="8"/>
         <v>6.3338533541341686</v>
       </c>
       <c r="H158" s="9" t="s">
@@ -6421,7 +6420,7 @@
         <v>300.2</v>
       </c>
       <c r="K158" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B158, $C$2:$C$979, C158, $D$2:$D$979, D158, $E$2:$E$979, E158) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6445,7 +6444,7 @@
         <v>9</v>
       </c>
       <c r="G159">
-        <f>((E159-I159)/E159)*100</f>
+        <f t="shared" si="8"/>
         <v>6.4199395770392753</v>
       </c>
       <c r="H159" s="9" t="s">
@@ -6455,7 +6454,7 @@
         <v>1239</v>
       </c>
       <c r="K159" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B159, $C$2:$C$979, C159, $D$2:$D$979, D159, $E$2:$E$979, E159) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6479,7 +6478,7 @@
         <v>9</v>
       </c>
       <c r="G160">
-        <f>((E160-I160)/E160)*100</f>
+        <f t="shared" si="8"/>
         <v>6.6011235955056176</v>
       </c>
       <c r="H160" s="9" t="s">
@@ -6489,7 +6488,7 @@
         <v>1330</v>
       </c>
       <c r="K160" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B160, $C$2:$C$979, C160, $D$2:$D$979, D160, $E$2:$E$979, E160) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6513,7 +6512,7 @@
         <v>9</v>
       </c>
       <c r="G161">
-        <f>((E161-I161)/E161)*100</f>
+        <f t="shared" si="8"/>
         <v>6.7632850241545892</v>
       </c>
       <c r="H161" s="9" t="s">
@@ -6523,7 +6522,7 @@
         <v>289.5</v>
       </c>
       <c r="K161" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B161, $C$2:$C$979, C161, $D$2:$D$979, D161, $E$2:$E$979, E161) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6547,7 +6546,7 @@
         <v>9</v>
       </c>
       <c r="G162">
-        <f>((E162-I162)/E162)*100</f>
+        <f t="shared" ref="G162:G187" si="10">((E162-I162)/E162)*100</f>
         <v>6.8620178041543021</v>
       </c>
       <c r="H162" s="9" t="s">
@@ -6557,7 +6556,7 @@
         <v>2511</v>
       </c>
       <c r="K162" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B162, $C$2:$C$979, C162, $D$2:$D$979, D162, $E$2:$E$979, E162) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="K162:K187" si="11">IF(COUNTIFS( $B$2:$B$979, B162, $C$2:$C$979, C162, $D$2:$D$979, D162, $E$2:$E$979, E162) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -6581,7 +6580,7 @@
         <v>9</v>
       </c>
       <c r="G163">
-        <f>((E163-I163)/E163)*100</f>
+        <f t="shared" si="10"/>
         <v>6.9140975755761751</v>
       </c>
       <c r="H163" s="9" t="s">
@@ -6591,7 +6590,7 @@
         <v>3110</v>
       </c>
       <c r="K163" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B163, $C$2:$C$979, C163, $D$2:$D$979, D163, $E$2:$E$979, E163) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6615,7 +6614,7 @@
         <v>9</v>
       </c>
       <c r="G164">
-        <f>((E164-I164)/E164)*100</f>
+        <f t="shared" si="10"/>
         <v>6.962025316455696</v>
       </c>
       <c r="H164" s="9" t="s">
@@ -6625,7 +6624,7 @@
         <v>735</v>
       </c>
       <c r="K164" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B164, $C$2:$C$979, C164, $D$2:$D$979, D164, $E$2:$E$979, E164) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6649,7 +6648,7 @@
         <v>9</v>
       </c>
       <c r="G165">
-        <f>((E165-I165)/E165)*100</f>
+        <f t="shared" si="10"/>
         <v>7.0841889117043113</v>
       </c>
       <c r="H165" s="9" t="s">
@@ -6659,7 +6658,7 @@
         <v>905</v>
       </c>
       <c r="K165" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B165, $C$2:$C$979, C165, $D$2:$D$979, D165, $E$2:$E$979, E165) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6683,7 +6682,7 @@
         <v>9</v>
       </c>
       <c r="G166">
-        <f>((E166-I166)/E166)*100</f>
+        <f t="shared" si="10"/>
         <v>7.3486328125</v>
       </c>
       <c r="H166" s="9" t="s">
@@ -6693,7 +6692,7 @@
         <v>948.75</v>
       </c>
       <c r="K166" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B166, $C$2:$C$979, C166, $D$2:$D$979, D166, $E$2:$E$979, E166) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6717,7 +6716,7 @@
         <v>9</v>
       </c>
       <c r="G167">
-        <f>((E167-I167)/E167)*100</f>
+        <f t="shared" si="10"/>
         <v>7.6838235294117654</v>
       </c>
       <c r="H167" s="9" t="s">
@@ -6727,7 +6726,7 @@
         <v>2511</v>
       </c>
       <c r="K167" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B167, $C$2:$C$979, C167, $D$2:$D$979, D167, $E$2:$E$979, E167) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6751,7 +6750,7 @@
         <v>9</v>
       </c>
       <c r="G168">
-        <f>((E168-I168)/E168)*100</f>
+        <f t="shared" si="10"/>
         <v>7.8025477707006363</v>
       </c>
       <c r="H168" s="9" t="s">
@@ -6761,7 +6760,7 @@
         <v>289.5</v>
       </c>
       <c r="K168" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B168, $C$2:$C$979, C168, $D$2:$D$979, D168, $E$2:$E$979, E168) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6785,7 +6784,7 @@
         <v>9</v>
       </c>
       <c r="G169">
-        <f>((E169-I169)/E169)*100</f>
+        <f t="shared" si="10"/>
         <v>7.8477690288713919</v>
       </c>
       <c r="H169" s="9" t="s">
@@ -6795,7 +6794,7 @@
         <v>3511</v>
       </c>
       <c r="K169" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B169, $C$2:$C$979, C169, $D$2:$D$979, D169, $E$2:$E$979, E169) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6819,7 +6818,7 @@
         <v>9</v>
       </c>
       <c r="G170">
-        <f>((E170-I170)/E170)*100</f>
+        <f t="shared" si="10"/>
         <v>8.160377358490571</v>
       </c>
       <c r="H170" s="9" t="s">
@@ -6829,7 +6828,7 @@
         <v>389.4</v>
       </c>
       <c r="K170" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B170, $C$2:$C$979, C170, $D$2:$D$979, D170, $E$2:$E$979, E170) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6853,7 +6852,7 @@
         <v>9</v>
       </c>
       <c r="G171">
-        <f>((E171-I171)/E171)*100</f>
+        <f t="shared" si="10"/>
         <v>8.1609195402298855</v>
       </c>
       <c r="H171" s="9" t="s">
@@ -6863,7 +6862,7 @@
         <v>399.5</v>
       </c>
       <c r="K171" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B171, $C$2:$C$979, C171, $D$2:$D$979, D171, $E$2:$E$979, E171) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6887,7 +6886,7 @@
         <v>9</v>
       </c>
       <c r="G172">
-        <f>((E172-I172)/E172)*100</f>
+        <f t="shared" si="10"/>
         <v>8.1818181818181817</v>
       </c>
       <c r="H172" s="9" t="s">
@@ -6897,7 +6896,7 @@
         <v>202</v>
       </c>
       <c r="K172" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B172, $C$2:$C$979, C172, $D$2:$D$979, D172, $E$2:$E$979, E172) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6921,7 +6920,7 @@
         <v>9</v>
       </c>
       <c r="G173">
-        <f>((E173-I173)/E173)*100</f>
+        <f t="shared" si="10"/>
         <v>8.1847389558232919</v>
       </c>
       <c r="H173" s="9" t="s">
@@ -6931,7 +6930,7 @@
         <v>228.62</v>
       </c>
       <c r="K173" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B173, $C$2:$C$979, C173, $D$2:$D$979, D173, $E$2:$E$979, E173) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6955,7 +6954,7 @@
         <v>9</v>
       </c>
       <c r="G174">
-        <f>((E174-I174)/E174)*100</f>
+        <f t="shared" si="10"/>
         <v>8.2150101419878307</v>
       </c>
       <c r="H174" s="9" t="s">
@@ -6965,7 +6964,7 @@
         <v>905</v>
       </c>
       <c r="K174" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B174, $C$2:$C$979, C174, $D$2:$D$979, D174, $E$2:$E$979, E174) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6989,7 +6988,7 @@
         <v>9</v>
       </c>
       <c r="G175">
-        <f>((E175-I175)/E175)*100</f>
+        <f t="shared" si="10"/>
         <v>8.544726301735647</v>
       </c>
       <c r="H175" s="9" t="s">
@@ -6999,7 +6998,7 @@
         <v>685</v>
       </c>
       <c r="K175" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B175, $C$2:$C$979, C175, $D$2:$D$979, D175, $E$2:$E$979, E175) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7023,7 +7022,7 @@
         <v>9</v>
       </c>
       <c r="G176">
-        <f>((E176-I176)/E176)*100</f>
+        <f t="shared" si="10"/>
         <v>8.6770833333333286</v>
       </c>
       <c r="H176" s="9" t="s">
@@ -7033,7 +7032,7 @@
         <v>438.35</v>
       </c>
       <c r="K176" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B176, $C$2:$C$979, C176, $D$2:$D$979, D176, $E$2:$E$979, E176) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7057,7 +7056,7 @@
         <v>9</v>
       </c>
       <c r="G177">
-        <f>((E177-I177)/E177)*100</f>
+        <f t="shared" si="10"/>
         <v>8.6964160224877016</v>
       </c>
       <c r="H177" s="9" t="s">
@@ -7067,7 +7066,7 @@
         <v>2598.5</v>
       </c>
       <c r="K177" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B177, $C$2:$C$979, C177, $D$2:$D$979, D177, $E$2:$E$979, E177) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7091,7 +7090,7 @@
         <v>9</v>
       </c>
       <c r="G178">
-        <f>((E178-I178)/E178)*100</f>
+        <f t="shared" si="10"/>
         <v>8.9622641509433958</v>
       </c>
       <c r="H178" s="9" t="s">
@@ -7101,7 +7100,7 @@
         <v>289.5</v>
       </c>
       <c r="K178" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B178, $C$2:$C$979, C178, $D$2:$D$979, D178, $E$2:$E$979, E178) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7125,7 +7124,7 @@
         <v>9</v>
       </c>
       <c r="G179">
-        <f>((E179-I179)/E179)*100</f>
+        <f t="shared" si="10"/>
         <v>9.0000000000000071</v>
       </c>
       <c r="H179" s="9" t="s">
@@ -7135,7 +7134,7 @@
         <v>208.39</v>
       </c>
       <c r="K179" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B179, $C$2:$C$979, C179, $D$2:$D$979, D179, $E$2:$E$979, E179) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7159,7 +7158,7 @@
         <v>9</v>
       </c>
       <c r="G180">
-        <f>((E180-I180)/E180)*100</f>
+        <f t="shared" si="10"/>
         <v>9.1365461847389557</v>
       </c>
       <c r="H180" s="9" t="s">
@@ -7169,7 +7168,7 @@
         <v>905</v>
       </c>
       <c r="K180" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B180, $C$2:$C$979, C180, $D$2:$D$979, D180, $E$2:$E$979, E180) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7193,7 +7192,7 @@
         <v>9</v>
       </c>
       <c r="G181">
-        <f>((E181-I181)/E181)*100</f>
+        <f t="shared" si="10"/>
         <v>9.2476489028213162</v>
       </c>
       <c r="H181" s="9" t="s">
@@ -7203,7 +7202,7 @@
         <v>289.5</v>
       </c>
       <c r="K181" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B181, $C$2:$C$979, C181, $D$2:$D$979, D181, $E$2:$E$979, E181) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7227,7 +7226,7 @@
         <v>9</v>
       </c>
       <c r="G182">
-        <f>((E182-I182)/E182)*100</f>
+        <f t="shared" si="10"/>
         <v>9.3501805054151621</v>
       </c>
       <c r="H182" s="9" t="s">
@@ -7237,7 +7236,7 @@
         <v>2511</v>
       </c>
       <c r="K182" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B182, $C$2:$C$979, C182, $D$2:$D$979, D182, $E$2:$E$979, E182) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7261,7 +7260,7 @@
         <v>9</v>
       </c>
       <c r="G183">
-        <f>((E183-I183)/E183)*100</f>
+        <f t="shared" si="10"/>
         <v>9.6806387225548907</v>
       </c>
       <c r="H183" s="9" t="s">
@@ -7271,7 +7270,7 @@
         <v>905</v>
       </c>
       <c r="K183" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B183, $C$2:$C$979, C183, $D$2:$D$979, D183, $E$2:$E$979, E183) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7295,7 +7294,7 @@
         <v>9</v>
       </c>
       <c r="G184">
-        <f>((E184-I184)/E184)*100</f>
+        <f t="shared" si="10"/>
         <v>10.371517027863778</v>
       </c>
       <c r="H184" s="9" t="s">
@@ -7305,7 +7304,7 @@
         <v>289.5</v>
       </c>
       <c r="K184" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B184, $C$2:$C$979, C184, $D$2:$D$979, D184, $E$2:$E$979, E184) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7329,7 +7328,7 @@
         <v>9</v>
       </c>
       <c r="G185">
-        <f>((E185-I185)/E185)*100</f>
+        <f t="shared" si="10"/>
         <v>11.265182186234814</v>
       </c>
       <c r="H185" s="9" t="s">
@@ -7339,7 +7338,7 @@
         <v>438.35</v>
       </c>
       <c r="K185" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B185, $C$2:$C$979, C185, $D$2:$D$979, D185, $E$2:$E$979, E185) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7363,7 +7362,7 @@
         <v>9</v>
       </c>
       <c r="G186" t="e">
-        <f>((E186-I186)/E186)*100</f>
+        <f t="shared" si="10"/>
         <v>#N/A</v>
       </c>
       <c r="H186" s="9" t="s">
@@ -7373,7 +7372,7 @@
         <v>#N/A</v>
       </c>
       <c r="K186" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B186, $C$2:$C$979, C186, $D$2:$D$979, D186, $E$2:$E$979, E186) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7397,7 +7396,7 @@
         <v>5</v>
       </c>
       <c r="G187" t="e">
-        <f>((E187-I187)/E187)*100</f>
+        <f t="shared" si="10"/>
         <v>#VALUE!</v>
       </c>
       <c r="H187" s="9" t="s">
@@ -7408,7 +7407,7 @@
       </c>
       <c r="J187" s="8"/>
       <c r="K187" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$979, B187, $C$2:$C$979, C187, $D$2:$D$979, D187, $E$2:$E$979, E187) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="11"/>
         <v>Unique</v>
       </c>
     </row>

</xml_diff>